<commit_message>
set threshold for definition tables to 0
</commit_message>
<xml_diff>
--- a/scripts/input/threshold.xlsx
+++ b/scripts/input/threshold.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PostEx-Waleed\Desktop\DockerImage\Airflow_Docker\scripts\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A124C39-C3BE-44D7-A548-CB13C03F8D08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1FD5AFB-808E-4D4B-A99B-D138AFAA173F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{073B13C2-E5F2-4830-92FA-1DE34A568199}"/>
   </bookViews>
@@ -7944,7 +7944,7 @@
         <v>55</v>
       </c>
       <c r="B549" s="5">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="550" spans="1:2">
@@ -7952,7 +7952,7 @@
         <v>56</v>
       </c>
       <c r="B550" s="3">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="551" spans="1:2">
@@ -8928,7 +8928,7 @@
         <v>700</v>
       </c>
       <c r="B672" s="5">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="673" spans="1:2">
@@ -9176,7 +9176,7 @@
         <v>25</v>
       </c>
       <c r="B703" s="5">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="704" spans="1:2">
@@ -9184,7 +9184,7 @@
         <v>26</v>
       </c>
       <c r="B704" s="3">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="705" spans="1:2">
@@ -10120,7 +10120,7 @@
         <v>27</v>
       </c>
       <c r="B821" s="5">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="822" spans="1:2">
@@ -10128,7 +10128,7 @@
         <v>28</v>
       </c>
       <c r="B822" s="3">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="823" spans="1:2">
@@ -10808,7 +10808,7 @@
         <v>29</v>
       </c>
       <c r="B907" s="5">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="908" spans="1:2">
@@ -10816,7 +10816,7 @@
         <v>30</v>
       </c>
       <c r="B908" s="3">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="909" spans="1:2">

</xml_diff>